<commit_message>
Update first-company core, remove promotion charges and add balance sweep evidence
</commit_message>
<xml_diff>
--- a/config/game_config.xlsx
+++ b/config/game_config.xlsx
@@ -397,12 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C145"/>
-  <cols>
-    <col min="1" max="1" width="48.83203125" customWidth="1"/>
-    <col min="2" max="2" width="70.83203125" customWidth="1"/>
-    <col min="3" max="3" width="55.83203125" customWidth="1"/>
-  </cols>
+  <dimension ref="A1:C152"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -475,7 +470,7 @@
         <v>time.dayDuration</v>
       </c>
       <c r="B7">
-        <v>60</v>
+        <v>180</v>
       </c>
       <c r="C7" t="str">
         <v>time.dayDuration</v>
@@ -585,7 +580,7 @@
         <v>economy.baseWorkSpeed</v>
       </c>
       <c r="B17">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="C17" t="str">
         <v>economy.baseWorkSpeed</v>
@@ -596,7 +591,7 @@
         <v>economy.baseQuality</v>
       </c>
       <c r="B18">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="C18" t="str">
         <v>economy.baseQuality</v>
@@ -1080,7 +1075,7 @@
         <v>ranks</v>
       </c>
       <c r="B62" t="str">
-        <v>[{"name":"新人","promotionCost":0,"workloadMultiplier":1,"rewardMultiplier":1,"qualityMultiplier":1,"projectChance":0.16,"recommendedSpeed":20,"recommendedQuality":10,"maxOverdueAllowed":0,"rankEscapeResistance":0},{"name":"一般員工","promotionCost":220,"workloadMultiplier":1.25,"rewardMultiplier":2.2,"qualityMultiplier":1.2,"projectChance":0.22,"recommendedSpeed":30,"recommendedQuality":18,"maxOverdueAllowed":3,"rankEscapeResistance":4},{"name":"資深員工","promotionCost":900,"workloadMultiplier":1.7,"rewardMultiplier":5,"qualityMultiplier":1.5,"projectChance":0.3,"recommendedSpeed":45,"recommendedQuality":28,"maxOverdueAllowed":2,"rankEscapeResistance":9},{"name":"主管","promotionCost":2800,"workloadMultiplier":2.2,"rewardMultiplier":11,"qualityMultiplier":1.8,"projectChance":0.4,"recommendedSpeed":65,"recommendedQuality":40,"maxOverdueAllowed":1,"rankEscapeResistance":14},{"name":"經理","promotionCost":9000,"workloadMultiplier":3,"rewardMultiplier":25,"qualityMultiplier":2.2,"projectChance":0.5,"recommendedSpeed":90,"recommendedQuality":55,"maxOverdueAllowed":0,"rankEscapeResistance":20}]</v>
+        <v>[{"name":"新人","promotionCost":0,"workloadMultiplier":1,"rewardMultiplier":1,"qualityMultiplier":1,"projectChance":0.16,"recommendedSpeed":10,"recommendedQuality":6,"maxOverdueAllowed":0,"rankEscapeResistance":0},{"name":"一般員工","promotionCost":220,"workloadMultiplier":1.25,"rewardMultiplier":2.2,"qualityMultiplier":1.2,"projectChance":0.22,"recommendedSpeed":20,"recommendedQuality":12,"maxOverdueAllowed":3,"rankEscapeResistance":4},{"name":"資深員工","promotionCost":900,"workloadMultiplier":1.7,"rewardMultiplier":5,"qualityMultiplier":1.5,"projectChance":0.3,"recommendedSpeed":40,"recommendedQuality":24,"maxOverdueAllowed":2,"rankEscapeResistance":9},{"name":"主管","promotionCost":2800,"workloadMultiplier":2.2,"rewardMultiplier":11,"qualityMultiplier":1.8,"projectChance":0.4,"recommendedSpeed":80,"recommendedQuality":48,"maxOverdueAllowed":1,"rankEscapeResistance":14},{"name":"經理","promotionCost":9000,"workloadMultiplier":3,"rewardMultiplier":25,"qualityMultiplier":2.2,"projectChance":0.5,"recommendedSpeed":160,"recommendedQuality":96,"maxOverdueAllowed":0,"rankEscapeResistance":20}]</v>
       </c>
       <c r="C62" t="str">
         <v>ranks</v>
@@ -1960,7 +1955,7 @@
         <v>promotionQualification.requirements</v>
       </c>
       <c r="B142" t="str">
-        <v>[{"efficiency":26,"quality":16},{"efficiency":38,"quality":24},{"efficiency":55,"quality":34},{"efficiency":78,"quality":48}]</v>
+        <v>[{"efficiency":20,"quality":12},{"efficiency":40,"quality":24},{"efficiency":80,"quality":48},{"efficiency":160,"quality":96}]</v>
       </c>
       <c r="C142" t="str">
         <v>Promotion V1 PROVISIONAL</v>
@@ -1999,9 +1994,86 @@
         <v>Promotion V1 PROVISIONAL</v>
       </c>
     </row>
+    <row r="146">
+      <c r="A146" t="str">
+        <v>time.sleepTimeAcceleration</v>
+      </c>
+      <c r="B146">
+        <v>60</v>
+      </c>
+      <c r="C146" t="str">
+        <v>First Company Incremental V1 · PROVISIONAL</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="str">
+        <v>promotionAssignment.workloadFactor</v>
+      </c>
+      <c r="B147">
+        <v>1.2</v>
+      </c>
+      <c r="C147" t="str">
+        <v>First Company Incremental V1 · PROVISIONAL</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="str">
+        <v>promotionAssignment.failedCompletionReward</v>
+      </c>
+      <c r="B148">
+        <v>0</v>
+      </c>
+      <c r="C148" t="str">
+        <v>First Company Incremental V1 · PROVISIONAL</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="str">
+        <v>work.workloadTierCenters</v>
+      </c>
+      <c r="B149" t="str">
+        <v>[70,140,280,560,1120]</v>
+      </c>
+      <c r="C149" t="str">
+        <v>First Company Incremental V1 · PROVISIONAL</v>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="str">
+        <v>work.templateWorkloadReference</v>
+      </c>
+      <c r="B150">
+        <v>100</v>
+      </c>
+      <c r="C150" t="str">
+        <v>First Company Incremental V1 · PROVISIONAL</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="str">
+        <v>work.templateVariationMin</v>
+      </c>
+      <c r="B151">
+        <v>0.75</v>
+      </c>
+      <c r="C151" t="str">
+        <v>First Company Incremental V1 · PROVISIONAL</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="str">
+        <v>work.templateVariationMax</v>
+      </c>
+      <c r="B152">
+        <v>1.4</v>
+      </c>
+      <c r="C152" t="str">
+        <v>First Company Incremental V1 · PROVISIONAL</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C145"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C152"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>